<commit_message>
Caso COL18 completo, barridos y app Streamlit inicial
Modelo
- Bloque hidraulico completo: 18 embalses + 4 filo de agua
- Restricciones huerfanas corregidas (hid_lim_caudal, hid_lim_vert, hid_rampa_sub)
- Penalizacion de vertimiento para romper degeneracion
- Banda de cierre de volumen configurable (tol_volumen_final = 0.15)

Resultados COL18
- E0-E3 a 168 h: ninguna tecnologia instalada a ningun nivel de costo
- Barrido de 24 puntos: objetivo invariante dentro de la tolerancia del solver
- Biseccion: el BESS no entra ni con costo de inversion nulo
- Causa: margen hidraulico en 161 de 168 h; ningun embalse con holgura
  simultanea de potencia y volumen
- Validacion contra XM: r = 0.83 en generacion semanal por embalse

Otros
- Streamlit inicial
- Rutas actualizadas de 04_Outputs a 03_Outputs

Siguiente: sistema de 120 nodos para recuperar los 173 corredores
internos descartados en la agregacion por subareas
</commit_message>
<xml_diff>
--- a/01_Data/03_Test_Cases/Colombian system/caso_COL18_E0_168h.xlsx
+++ b/01_Data/03_Test_Cases/Colombian system/caso_COL18_E0_168h.xlsx
@@ -785,7 +785,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -8348,6 +8347,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -8516,7 +8516,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -19673,7 +19672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -19928,11 +19927,26 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>Banda del cierre de volumen: |V_T - V_init| &lt;= tol*(Vmax-Vmin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>costo_vertimiento</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Regularizacion del vertimiento [USD por m3/s y hora]. No es un costo real.</t>
         </is>
       </c>
     </row>
@@ -20246,10 +20260,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="6"/>
+    <col width="10" customWidth="1" min="1" max="6"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -20267,739 +20288,961 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>desde</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>hasta</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>capacidad_termica</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>capacidad</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>origen_capacidad</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>nodo</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>nodo</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>p.u.</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>p.u.</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>l1</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>ANT</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>BOG</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" t="n">
         <v>0.0018431712</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" t="n">
         <v>0.026072208</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" t="n">
         <v>1649.778394209355</v>
       </c>
+      <c r="G6" t="n">
+        <v>1649.778394209355</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>l2</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>ANT</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>CQR</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" t="n">
         <v>0.0005677017783951298</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" t="n">
         <v>0.006457710663587037</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" t="n">
         <v>4754.82953241286</v>
       </c>
+      <c r="G7" t="n">
+        <v>4754.82953241286</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>UPME p.317 (circuito SC-LV) + termico (9 circuitos)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>l3</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>ANT</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>CER</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" t="n">
         <v>0.0003440353363085841</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" t="n">
         <v>0.00445599503825384</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" t="n">
         <v>6693.038359406769</v>
       </c>
+      <c r="G8" t="n">
+        <v>6693.038359406769</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>l4</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>ANT</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>SAN</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" t="n">
         <v>0.0007685703245136628</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" t="n">
         <v>0.00875226955914961</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" t="n">
         <v>3385.920344387896</v>
       </c>
+      <c r="G9" t="n">
+        <v>3385.920344387896</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>l5</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>ARA</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>SAN</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" t="n">
         <v>0.008080170132325143</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" t="n">
         <v>0.07752758034026465</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" t="n">
         <v>346.1849949087915</v>
       </c>
+      <c r="G10" t="n">
+        <v>346.1849949087915</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>l6</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>ATL</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>BOL</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" t="n">
         <v>0.000541051702307867</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" t="n">
         <v>0.006199517060556735</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" t="n">
         <v>3579.558668862747</v>
       </c>
+      <c r="G11" t="n">
+        <v>3579.558668862747</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>l7</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>ATL</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>CSU</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" t="n">
         <v>0.0009797041718811791</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" t="n">
         <v>0.01214247572075158</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" t="n">
         <v>4088.265156988669</v>
       </c>
+      <c r="G12" t="n">
+        <v>4088.265156988669</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>l8</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>ATL</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>GCM</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" t="n">
         <v>0.005675323621960651</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" t="n">
         <v>0.03180369317142009</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" t="n">
         <v>970.4198679288653</v>
       </c>
+      <c r="G13" t="n">
+        <v>970.4198679288653</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>l9</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>BOG</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>BYC</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" t="n">
         <v>0.00543959168241966</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" t="n">
         <v>0.05316762192816636</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" t="n">
         <v>813.4749822827987</v>
       </c>
+      <c r="G14" t="n">
+        <v>813.4749822827987</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>l10</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>BOG</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>CQR</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" t="n">
         <v>0.001077894408851415</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" t="n">
         <v>0.01204469736581769</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" t="n">
         <v>2268.121412751985</v>
       </c>
+      <c r="G15" t="n">
+        <v>2268.121412751985</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>l11</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>BOG</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>HTO</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" t="n">
         <v>0.00438542995617135</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" t="n">
         <v>0.03956723438960581</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" t="n">
         <v>769.0776765690694</v>
       </c>
+      <c r="G16" t="n">
+        <v>769.0776765690694</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>l12</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>BOG</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>MET</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" t="n">
         <v>0.001296732471385508</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" t="n">
         <v>0.01509439111011182</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" t="n">
         <v>2374.596980925328</v>
       </c>
+      <c r="G17" t="n">
+        <v>2374.596980925328</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>l13</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>BOL</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>CSU</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" t="n">
         <v>0.01441566115702479</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" t="n">
         <v>0.08854997107438016</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" t="n">
         <v>435.922547248935</v>
       </c>
+      <c r="G18" t="n">
+        <v>435.922547248935</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>l14</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>BOL</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>GCM</t>
         </is>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="D19" t="n">
         <v>0.0015801264</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" t="n">
         <v>0.0222817824</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" t="n">
         <v>2144.27889977027</v>
       </c>
+      <c r="G19" t="n">
+        <v>2144.27889977027</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>l15</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>BYC</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>SAN</t>
         </is>
       </c>
-      <c r="D20" s="5" t="n">
+      <c r="D20" t="n">
         <v>0.008170244811082653</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" t="n">
         <v>0.06926589199970112</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" t="n">
         <v>658.6615517470284</v>
       </c>
+      <c r="G20" t="n">
+        <v>658.6615517470284</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>l16</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>CQR</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>VAL</t>
         </is>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D21" t="n">
         <v>0.0005306751075759304</v>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E21" t="n">
         <v>0.005494828273578538</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" t="n">
         <v>1155.501349235845</v>
       </c>
+      <c r="G21" t="n">
+        <v>1155.501349235845</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>l17</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>CAQ</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
       </c>
-      <c r="D22" s="5" t="n">
+      <c r="D22" t="n">
         <v>0.004725727788279773</v>
       </c>
-      <c r="E22" s="5" t="n">
+      <c r="E22" t="n">
         <v>0.03510943289224953</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" t="n">
         <v>563.2975636375502</v>
       </c>
+      <c r="G22" t="n">
+        <v>563.2975636375502</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>l18</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>CAQ</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>HTO</t>
         </is>
       </c>
-      <c r="D23" s="5" t="n">
+      <c r="D23" t="n">
         <v>0.00746276370510397</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" t="n">
         <v>0.05598634026465028</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" t="n">
         <v>550.1512980081025</v>
       </c>
+      <c r="G23" t="n">
+        <v>550.1512980081025</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>l19</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>CAQ</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="D24" s="5" t="n">
+      <c r="D24" t="n">
         <v>0.01286747069943289</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="E24" t="n">
         <v>0.09818617769376183</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" t="n">
         <v>550.9480413795841</v>
       </c>
+      <c r="G24" t="n">
+        <v>550.9480413795841</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>l20</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>HTO</t>
         </is>
       </c>
-      <c r="D25" s="5" t="n">
+      <c r="D25" t="n">
         <v>0.002269156759125412</v>
       </c>
-      <c r="E25" s="5" t="n">
+      <c r="E25" t="n">
         <v>0.01755093702254853</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" t="n">
         <v>986.8261390698508</v>
       </c>
+      <c r="G25" t="n">
+        <v>986.8261390698508</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>l21</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="D26" s="5" t="n">
+      <c r="D26" t="n">
         <v>0.01244615500945179</v>
       </c>
-      <c r="E26" s="5" t="n">
+      <c r="E26" t="n">
         <v>0.07344083931947069</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" t="n">
         <v>274.8764631611808</v>
       </c>
+      <c r="G26" t="n">
+        <v>274.8764631611808</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>l22</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>VAL</t>
         </is>
       </c>
-      <c r="D27" s="5" t="n">
+      <c r="D27" t="n">
         <v>0.002042286435992805</v>
       </c>
-      <c r="E27" s="5" t="n">
+      <c r="E27" t="n">
         <v>0.0187738215422143</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" t="n">
         <v>676.3251650765665</v>
       </c>
+      <c r="G27" t="n">
+        <v>676.3251650765665</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>l23</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>CER</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>CSU</t>
         </is>
       </c>
-      <c r="D28" s="5" t="n">
+      <c r="D28" t="n">
         <v>0.0003446098485410753</v>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="E28" t="n">
         <v>0.004798599373031993</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" t="n">
         <v>4852.559547816959</v>
       </c>
+      <c r="G28" t="n">
+        <v>4852.559547816959</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>l24</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>CSU</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>GCM</t>
         </is>
       </c>
-      <c r="D29" s="5" t="n">
+      <c r="D29" t="n">
         <v>0.0026140868</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E29" t="n">
         <v>0.0289875248</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" t="n">
         <v>2078.460969082652</v>
       </c>
+      <c r="G29" t="n">
+        <v>2078.460969082652</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>l25</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>GCM</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>NDS</t>
         </is>
       </c>
-      <c r="D30" s="5" t="n">
+      <c r="D30" t="n">
         <v>0.0010752</v>
       </c>
-      <c r="E30" s="5" t="n">
+      <c r="E30" t="n">
         <v>0.0239232</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" t="n">
         <v>2144.27889977027</v>
       </c>
+      <c r="G30" t="n">
+        <v>2144.27889977027</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>l26</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>NDS</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>SAN</t>
         </is>
       </c>
-      <c r="D31" s="5" t="n">
+      <c r="D31" t="n">
         <v>0.001305884247969807</v>
       </c>
-      <c r="E31" s="5" t="n">
+      <c r="E31" t="n">
         <v>0.01407934656508677</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" t="n">
         <v>2363.389511522908</v>
+      </c>
+      <c r="G31" t="n">
+        <v>2363.389511522908</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>termico</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -23272,7 +23515,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>

</xml_diff>